<commit_message>
Auto-generate blog post 2026-05-25
</commit_message>
<xml_diff>
--- a/GrowthMax-Keyword-Program.xlsx
+++ b/GrowthMax-Keyword-Program.xlsx
@@ -2187,12 +2187,12 @@
       </c>
       <c r="M21" s="5" t="inlineStr">
         <is>
-          <t>Spoke post — definitional; high AEO capture</t>
+          <t>Published</t>
         </is>
       </c>
       <c r="N21" s="5" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>/blog/ai-agent-vs-ai-assistant-vs-chatbot/</t>
         </is>
       </c>
       <c r="O21" s="5" t="inlineStr">
@@ -7528,7 +7528,12 @@
       <c r="G8" s="5" t="n"/>
       <c r="H8" s="5" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Published 2026-05-25</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>/blog/ai-agent-vs-ai-assistant-vs-chatbot/</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-generate blog post 2026-06-01
</commit_message>
<xml_diff>
--- a/GrowthMax-Keyword-Program.xlsx
+++ b/GrowthMax-Keyword-Program.xlsx
@@ -3192,12 +3192,12 @@
       </c>
       <c r="M36" s="5" t="inlineStr">
         <is>
-          <t>Published (same as K033)</t>
+          <t>Published</t>
         </is>
       </c>
       <c r="N36" s="5" t="inlineStr">
         <is>
-          <t>/blog/where-do-i-fit-crisis/</t>
+          <t>/blog/ai-adoption-metrics-that-actually-matter/</t>
         </is>
       </c>
       <c r="O36" s="5" t="inlineStr">
@@ -7601,7 +7601,12 @@
       <c r="G10" s="5" t="n"/>
       <c r="H10" s="5" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Published 2026-06-01</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>/blog/ai-adoption-metrics-that-actually-matter/</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-generate blog post 2026-06-08
</commit_message>
<xml_diff>
--- a/GrowthMax-Keyword-Program.xlsx
+++ b/GrowthMax-Keyword-Program.xlsx
@@ -2120,12 +2120,12 @@
       </c>
       <c r="M20" s="5" t="inlineStr">
         <is>
-          <t>Spoke post with diagram (SVG); link to pillar</t>
+          <t>Published</t>
         </is>
       </c>
       <c r="N20" s="5" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>/blog/ai-agent-architecture-explained-non-engineers/</t>
         </is>
       </c>
       <c r="O20" s="5" t="inlineStr">
@@ -7640,7 +7640,12 @@
       <c r="G11" s="5" t="n"/>
       <c r="H11" s="5" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Published 2026-06-08</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>/blog/ai-agent-architecture-explained-non-engineers/</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-generate blog post 2026-07-01
</commit_message>
<xml_diff>
--- a/GrowthMax-Keyword-Program.xlsx
+++ b/GrowthMax-Keyword-Program.xlsx
@@ -1249,12 +1249,12 @@
       </c>
       <c r="M7" s="5" t="inlineStr">
         <is>
-          <t>New 2,000-word spoke post with downloadable template</t>
+          <t>Published</t>
         </is>
       </c>
       <c r="N7" s="5" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>/blog/12-month-ai-transformation-roadmap/</t>
         </is>
       </c>
       <c r="O7" s="5" t="inlineStr">
@@ -7679,7 +7679,12 @@
       <c r="G12" s="5" t="n"/>
       <c r="H12" s="5" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Published 2026-07-01</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>/blog/12-month-ai-transformation-roadmap/</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-generate blog post 2026-07-03
</commit_message>
<xml_diff>
--- a/GrowthMax-Keyword-Program.xlsx
+++ b/GrowthMax-Keyword-Program.xlsx
@@ -2589,12 +2589,12 @@
       </c>
       <c r="M27" s="5" t="inlineStr">
         <is>
-          <t>Spoke with ranges and cost-driver breakdown</t>
+          <t>Published</t>
         </is>
       </c>
       <c r="N27" s="5" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>/blog/what-a-custom-ai-agent-costs-and-why/</t>
         </is>
       </c>
       <c r="O27" s="5" t="inlineStr">
@@ -7718,7 +7718,12 @@
       <c r="G13" s="5" t="n"/>
       <c r="H13" s="5" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Published 2026-07-03</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>/blog/what-a-custom-ai-agent-costs-and-why/</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-generate blog post 2026-07-06
</commit_message>
<xml_diff>
--- a/GrowthMax-Keyword-Program.xlsx
+++ b/GrowthMax-Keyword-Program.xlsx
@@ -2388,12 +2388,12 @@
       </c>
       <c r="M24" s="5" t="inlineStr">
         <is>
-          <t>Use-case spoke post</t>
+          <t>Published</t>
         </is>
       </c>
       <c r="N24" s="5" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>/blog/ai-agents-for-operations-teams/</t>
         </is>
       </c>
       <c r="O24" s="5" t="inlineStr">
@@ -7757,7 +7757,12 @@
       <c r="G14" s="5" t="n"/>
       <c r="H14" s="5" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Published 2026-07-06</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>/blog/ai-agents-for-operations-teams/</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-generate blog post 2026-07-08
</commit_message>
<xml_diff>
--- a/GrowthMax-Keyword-Program.xlsx
+++ b/GrowthMax-Keyword-Program.xlsx
@@ -1316,12 +1316,12 @@
       </c>
       <c r="M8" s="5" t="inlineStr">
         <is>
-          <t>Spoke post + interactive checklist (use Typeform/Tally)</t>
+          <t>Published</t>
         </is>
       </c>
       <c r="N8" s="5" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>/blog/ai-readiness-assessment/</t>
         </is>
       </c>
       <c r="O8" s="5" t="inlineStr">
@@ -7796,7 +7796,12 @@
       <c r="G15" s="5" t="n"/>
       <c r="H15" s="5" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Published 2026-07-08</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>/blog/ai-readiness-assessment/</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-generate blog post 2026-07-10
</commit_message>
<xml_diff>
--- a/GrowthMax-Keyword-Program.xlsx
+++ b/GrowthMax-Keyword-Program.xlsx
@@ -3795,12 +3795,12 @@
       </c>
       <c r="M45" s="5" t="inlineStr">
         <is>
-          <t>Spoke post — low competition, high-value persona</t>
+          <t>Published</t>
         </is>
       </c>
       <c r="N45" s="5" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>/blog/guide-to-ai-training-for-executives/</t>
         </is>
       </c>
       <c r="O45" s="5" t="inlineStr">
@@ -7835,7 +7835,12 @@
       <c r="G16" s="5" t="n"/>
       <c r="H16" s="5" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Published 2026-07-10</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>/blog/guide-to-ai-training-for-executives/</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-generate blog post 2026-07-15
</commit_message>
<xml_diff>
--- a/GrowthMax-Keyword-Program.xlsx
+++ b/GrowthMax-Keyword-Program.xlsx
@@ -4532,12 +4532,12 @@
       </c>
       <c r="M56" s="5" t="inlineStr">
         <is>
-          <t>Spoke with nuanced POV</t>
+          <t>Published</t>
         </is>
       </c>
       <c r="N56" s="5" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>/blog/will-ai-replace-my-job/</t>
         </is>
       </c>
       <c r="O56" s="5" t="inlineStr">
@@ -7874,7 +7874,12 @@
       <c r="G17" s="5" t="n"/>
       <c r="H17" s="5" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Published 2026-07-15</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>/blog/will-ai-replace-my-job/</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-generate blog post 2026-07-17
</commit_message>
<xml_diff>
--- a/GrowthMax-Keyword-Program.xlsx
+++ b/GrowthMax-Keyword-Program.xlsx
@@ -2254,12 +2254,12 @@
       </c>
       <c r="M22" s="5" t="inlineStr">
         <is>
-          <t>Spoke post — covers SSO, data handling, audit trails</t>
+          <t>Published</t>
         </is>
       </c>
       <c r="N22" s="5" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>/blog/enterprise-ai-agent-security-buyers-checklist/</t>
         </is>
       </c>
       <c r="O22" s="5" t="inlineStr">
@@ -7913,7 +7913,12 @@
       <c r="G18" s="5" t="n"/>
       <c r="H18" s="5" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Published 2026-07-17</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>/blog/enterprise-ai-agent-security-buyers-checklist/</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-generate blog post 2026-07-22
</commit_message>
<xml_diff>
--- a/GrowthMax-Keyword-Program.xlsx
+++ b/GrowthMax-Keyword-Program.xlsx
@@ -2455,12 +2455,12 @@
       </c>
       <c r="M25" s="5" t="inlineStr">
         <is>
-          <t>Use-case spoke post</t>
+          <t>Published</t>
         </is>
       </c>
       <c r="N25" s="5" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>/blog/ai-agents-for-finance-teams/</t>
         </is>
       </c>
       <c r="O25" s="5" t="inlineStr">
@@ -7952,7 +7952,12 @@
       <c r="G19" s="5" t="n"/>
       <c r="H19" s="5" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Published 2026-07-22</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>/blog/ai-agents-for-finance-teams/</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-generate blog post 2026-07-24
</commit_message>
<xml_diff>
--- a/GrowthMax-Keyword-Program.xlsx
+++ b/GrowthMax-Keyword-Program.xlsx
@@ -1651,12 +1651,12 @@
       </c>
       <c r="M13" s="5" t="inlineStr">
         <is>
-          <t>Spoke post with scorecard</t>
+          <t>Published</t>
         </is>
       </c>
       <c r="N13" s="5" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>/blog/how-to-evaluate-ai-vendors-scorecard/</t>
         </is>
       </c>
       <c r="O13" s="5" t="inlineStr">
@@ -7991,7 +7991,12 @@
       <c r="G20" s="5" t="n"/>
       <c r="H20" s="5" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Published 2026-07-24</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>/blog/how-to-evaluate-ai-vendors-scorecard/</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-generate blog post 2026-07-27
</commit_message>
<xml_diff>
--- a/GrowthMax-Keyword-Program.xlsx
+++ b/GrowthMax-Keyword-Program.xlsx
@@ -4599,12 +4599,12 @@
       </c>
       <c r="M57" s="5" t="inlineStr">
         <is>
-          <t>Spoke post</t>
+          <t>Published</t>
         </is>
       </c>
       <c r="N57" s="5" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>/blog/human-in-the-loop-ai-enterprise/</t>
         </is>
       </c>
       <c r="O57" s="5" t="inlineStr">
@@ -8030,7 +8030,12 @@
       <c r="G21" s="5" t="n"/>
       <c r="H21" s="5" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Published 2026-07-27</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>/blog/human-in-the-loop-ai-enterprise/</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-generate blog post 2026-07-31
</commit_message>
<xml_diff>
--- a/GrowthMax-Keyword-Program.xlsx
+++ b/GrowthMax-Keyword-Program.xlsx
@@ -1455,7 +1455,7 @@
       </c>
       <c r="N10" s="5" t="inlineStr">
         <is>
-          <t>/blog/custom-ai-agents-vs-off-shelf-tools-when-to-build/</t>
+          <t>/blog/ai-governance-framework-enterprise/</t>
         </is>
       </c>
       <c r="O10" s="5" t="inlineStr">
@@ -8069,7 +8069,12 @@
       <c r="G22" s="5" t="n"/>
       <c r="H22" s="5" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Published 2026-07-31</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>/blog/ai-governance-framework-enterprise/</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-generate blog post 2026-08-03
</commit_message>
<xml_diff>
--- a/GrowthMax-Keyword-Program.xlsx
+++ b/GrowthMax-Keyword-Program.xlsx
@@ -1785,12 +1785,12 @@
       </c>
       <c r="M15" s="5" t="inlineStr">
         <is>
-          <t>Spoke post — uncommon angle, lower competition</t>
+          <t>Published</t>
         </is>
       </c>
       <c r="N15" s="5" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>/blog/ai-pilot-to-production-what-goes-wrong/</t>
         </is>
       </c>
       <c r="O15" s="5" t="inlineStr">
@@ -8108,7 +8108,12 @@
       <c r="G23" s="5" t="n"/>
       <c r="H23" s="5" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Published 2026-08-03</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>/blog/ai-pilot-to-production-what-goes-wrong/</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-generate blog post 2026-08-05
</commit_message>
<xml_diff>
--- a/GrowthMax-Keyword-Program.xlsx
+++ b/GrowthMax-Keyword-Program.xlsx
@@ -1723,7 +1723,7 @@
       </c>
       <c r="N14" s="5" t="inlineStr">
         <is>
-          <t>/blog/hidden-costs-ai-implementation-beyond-technology-budget/</t>
+          <t>/blog/ai-business-case-template/</t>
         </is>
       </c>
       <c r="O14" s="5" t="inlineStr">
@@ -8147,7 +8147,12 @@
       <c r="G24" s="5" t="n"/>
       <c r="H24" s="5" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Published 2026-08-05</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>/blog/ai-business-case-template/</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-generate blog post 2026-08-07
</commit_message>
<xml_diff>
--- a/GrowthMax-Keyword-Program.xlsx
+++ b/GrowthMax-Keyword-Program.xlsx
@@ -4063,12 +4063,12 @@
       </c>
       <c r="M49" s="5" t="inlineStr">
         <is>
-          <t>Spoke post</t>
+          <t>Published</t>
         </is>
       </c>
       <c r="N49" s="5" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>/blog/what-belongs-in-an-ai-literacy-curriculum/</t>
         </is>
       </c>
       <c r="O49" s="5" t="inlineStr">
@@ -8186,7 +8186,12 @@
       <c r="G25" s="5" t="n"/>
       <c r="H25" s="5" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Published 2026-08-07</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>/blog/what-belongs-in-an-ai-literacy-curriculum/</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-generate blog post 2026-08-10
</commit_message>
<xml_diff>
--- a/GrowthMax-Keyword-Program.xlsx
+++ b/GrowthMax-Keyword-Program.xlsx
@@ -3996,12 +3996,12 @@
       </c>
       <c r="M48" s="5" t="inlineStr">
         <is>
-          <t>Spoke post linking to both training solutions</t>
+          <t>Published</t>
         </is>
       </c>
       <c r="N48" s="5" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>/blog/how-to-upskill-your-workforce-on-ai/</t>
         </is>
       </c>
       <c r="O48" s="5" t="inlineStr">
@@ -8225,7 +8225,12 @@
       <c r="G26" s="5" t="n"/>
       <c r="H26" s="5" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Published 2026-08-10</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>/blog/how-to-upskill-your-workforce-on-ai/</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-generate blog post 2026-08-12
</commit_message>
<xml_diff>
--- a/GrowthMax-Keyword-Program.xlsx
+++ b/GrowthMax-Keyword-Program.xlsx
@@ -3130,7 +3130,7 @@
       </c>
       <c r="N35" s="5" t="inlineStr">
         <is>
-          <t>/blog/where-do-i-fit-crisis/</t>
+          <t>/blog/growthmax-ai-adoption-framework/</t>
         </is>
       </c>
       <c r="O35" s="5" t="inlineStr">
@@ -8264,7 +8264,12 @@
       <c r="G27" s="5" t="n"/>
       <c r="H27" s="5" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Published 2026-08-12</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>/blog/growthmax-ai-adoption-framework/</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-generate blog post 2026-08-14
</commit_message>
<xml_diff>
--- a/GrowthMax-Keyword-Program.xlsx
+++ b/GrowthMax-Keyword-Program.xlsx
@@ -1517,12 +1517,12 @@
       </c>
       <c r="M11" s="5" t="inlineStr">
         <is>
-          <t>Spoke post on structure, staffing, charter</t>
+          <t>Published</t>
         </is>
       </c>
       <c r="N11" s="5" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>/blog/ai-center-of-excellence-playbook/</t>
         </is>
       </c>
       <c r="O11" s="5" t="inlineStr">
@@ -8303,7 +8303,12 @@
       <c r="G28" s="5" t="n"/>
       <c r="H28" s="5" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Published 2026-08-14</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>/blog/ai-center-of-excellence-playbook/</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-generate blog post 2026-08-17
</commit_message>
<xml_diff>
--- a/GrowthMax-Keyword-Program.xlsx
+++ b/GrowthMax-Keyword-Program.xlsx
@@ -3527,12 +3527,12 @@
       </c>
       <c r="M41" s="5" t="inlineStr">
         <is>
-          <t>Spoke with downloadable template</t>
+          <t>Published</t>
         </is>
       </c>
       <c r="N41" s="5" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>/blog/ai-rollout-plan-your-team-will-actually-follow/</t>
         </is>
       </c>
       <c r="O41" s="5" t="inlineStr">
@@ -8342,7 +8342,12 @@
       <c r="G29" s="5" t="n"/>
       <c r="H29" s="5" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Published 2026-08-17</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>/blog/ai-rollout-plan-your-team-will-actually-follow/</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-generate blog post 2026-08-19
</commit_message>
<xml_diff>
--- a/GrowthMax-Keyword-Program.xlsx
+++ b/GrowthMax-Keyword-Program.xlsx
@@ -4130,12 +4130,12 @@
       </c>
       <c r="M50" s="5" t="inlineStr">
         <is>
-          <t>Spoke with framework</t>
+          <t>Published</t>
         </is>
       </c>
       <c r="N50" s="5" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>/blog/measuring-roi-on-enterprise-ai-training/</t>
         </is>
       </c>
       <c r="O50" s="5" t="inlineStr">
@@ -8381,7 +8381,12 @@
       <c r="G30" s="5" t="n"/>
       <c r="H30" s="5" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Published 2026-08-19</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>/blog/measuring-roi-on-enterprise-ai-training/</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-generate blog post 2026-09-08
</commit_message>
<xml_diff>
--- a/GrowthMax-Keyword-Program.xlsx
+++ b/GrowthMax-Keyword-Program.xlsx
@@ -1,19 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="3960" yWindow="3120" windowWidth="26720" windowHeight="17040" tabRatio="500" firstSheet="0" activeTab="7" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pillars" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Master Keywords" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AEO Questions" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Content Gaps" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Calendar (90-day)" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracking Setup" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quick Wins" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Overview" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Pillars" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Master Keywords" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="AEO Questions" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Content Gaps" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Calendar (90-day)" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Tracking Setup" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Quick Wins" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Master Keywords'!$A$4:$O$60</definedName>
@@ -1988,12 +1988,12 @@
       </c>
       <c r="M18" s="5" t="inlineStr">
         <is>
-          <t>Optimize H1 and meta; add enterprise-specific proof section</t>
+          <t>Published</t>
         </is>
       </c>
       <c r="N18" s="5" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>/blog/what-makes-an-ai-agent-enterprise-ready/</t>
         </is>
       </c>
       <c r="O18" s="5" t="inlineStr">
@@ -9166,7 +9166,12 @@
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Published 2026-09-08</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>/blog/what-makes-an-ai-agent-enterprise-ready/</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-generate blog post 2026-09-09
</commit_message>
<xml_diff>
--- a/GrowthMax-Keyword-Program.xlsx
+++ b/GrowthMax-Keyword-Program.xlsx
@@ -3663,12 +3663,12 @@
       </c>
       <c r="M43" s="5" t="inlineStr">
         <is>
-          <t>Add H2 targeting this; link from new literacy pillar</t>
+          <t>Published</t>
         </is>
       </c>
       <c r="N43" s="5" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>/blog/what-effective-enterprise-ai-training-actually-looks-like/</t>
         </is>
       </c>
       <c r="O43" s="5" t="inlineStr">
@@ -9209,7 +9209,12 @@
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Published 2026-09-09</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>/blog/what-effective-enterprise-ai-training-actually-looks-like/</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-generate blog post 2026-09-11
</commit_message>
<xml_diff>
--- a/GrowthMax-Keyword-Program.xlsx
+++ b/GrowthMax-Keyword-Program.xlsx
@@ -2055,12 +2055,12 @@
       </c>
       <c r="M19" s="5" t="inlineStr">
         <is>
-          <t>Add H2 + FAQ schema</t>
+          <t>Published</t>
         </is>
       </c>
       <c r="N19" s="5" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>/blog/how-enterprise-ai-agent-development-actually-works/</t>
         </is>
       </c>
       <c r="O19" s="5" t="inlineStr">
@@ -9252,7 +9252,12 @@
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Published 2026-09-11</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>/blog/how-enterprise-ai-agent-development-actually-works/</t>
         </is>
       </c>
     </row>

</xml_diff>